<commit_message>
fix(sample-data): rebuild underwriting sheets with correct column names
Replaced Term/FICO/DTI/PTI/Max Balance columns with what underwriting.py
actually reads: finance_type_name_nls, monthly_income_min, fico_min,
approval_high, dti_max, pti_ratio.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/sample/files_required/Underwriting_Grids_COMAP.xlsx
+++ b/backend/data/sample/files_required/Underwriting_Grids_COMAP.xlsx
@@ -425,83 +425,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>finance_type_name_nls</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>monthly_income_min</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DTI</t>
+          <t>fico_min</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>PTI</t>
+          <t>approval_high</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Max Balance</t>
+          <t>dti_max</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>pti_ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>120</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STD</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>600</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>500000</v>
       </c>
       <c r="E2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Standard guideline</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>180</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STD</t>
+        </is>
       </c>
       <c r="B3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C3" t="n">
         <v>680</v>
       </c>
-      <c r="C3" t="n">
-        <v>45</v>
-      </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>350000</v>
       </c>
       <c r="E3" t="n">
-        <v>400000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Extended term guideline</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STD</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>720</v>
+      </c>
+      <c r="D4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -1115,83 +1137,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>finance_type_name_nls</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>monthly_income_min</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DTI</t>
+          <t>fico_min</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>PTI</t>
+          <t>approval_high</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Max Balance</t>
+          <t>dti_max</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>pti_ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>120</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_STD</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>600</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>500000</v>
       </c>
       <c r="E2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Standard guideline</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>180</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_STD</t>
+        </is>
       </c>
       <c r="B3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C3" t="n">
         <v>680</v>
       </c>
-      <c r="C3" t="n">
-        <v>45</v>
-      </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>350000</v>
       </c>
       <c r="E3" t="n">
-        <v>400000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Extended term guideline</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_STD</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>720</v>
+      </c>
+      <c r="D4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HD</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>600</v>
+      </c>
+      <c r="D5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HD</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C6" t="n">
+        <v>680</v>
+      </c>
+      <c r="D6" t="n">
+        <v>350000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>43</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HD</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C7" t="n">
+        <v>720</v>
+      </c>
+      <c r="D7" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>38</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -1205,83 +1315,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>finance_type_name_nls</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>monthly_income_min</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DTI</t>
+          <t>fico_min</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>PTI</t>
+          <t>approval_high</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Max Balance</t>
+          <t>dti_max</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>pti_ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>120</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STDnotes</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>600</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>500000</v>
       </c>
       <c r="E2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Standard guideline</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>180</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STDnotes</t>
+        </is>
       </c>
       <c r="B3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C3" t="n">
         <v>680</v>
       </c>
-      <c r="C3" t="n">
-        <v>45</v>
-      </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>350000</v>
       </c>
       <c r="E3" t="n">
-        <v>400000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Extended term guideline</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FX3_SFY_STDnotes</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>720</v>
+      </c>
+      <c r="D4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -1295,83 +1427,105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Term</t>
+          <t>finance_type_name_nls</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>FICO</t>
+          <t>monthly_income_min</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>DTI</t>
+          <t>fico_min</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>PTI</t>
+          <t>approval_high</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Max Balance</t>
+          <t>dti_max</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>pti_ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>120</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HDnotes</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>600</v>
       </c>
       <c r="D2" t="n">
-        <v>22</v>
+        <v>500000</v>
       </c>
       <c r="E2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Standard guideline</t>
-        </is>
+        <v>50</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>180</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HDnotes</t>
+        </is>
       </c>
       <c r="B3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C3" t="n">
         <v>680</v>
       </c>
-      <c r="C3" t="n">
-        <v>45</v>
-      </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>350000</v>
       </c>
       <c r="E3" t="n">
-        <v>400000</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Extended term guideline</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FX3_PRIME_HDnotes</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C4" t="n">
+        <v>720</v>
+      </c>
+      <c r="D4" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>